<commit_message>
Refactor Google Maps link generation
- Use `urllib.parse` to generate proper URL encodings
- Update generation to use structured location dict mapping
- Exclude CEP in textual location string for Map routing robustness
- Add logic to fallback to exact coordinates based on original Geocoding success and confidence criteria

Co-authored-by: juniorchiodi <95029115+juniorchiodi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ENDERECOS-ROTA.xlsx
+++ b/ENDERECOS-ROTA.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -40,7 +43,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,12 +51,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -424,57 +436,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Logradouro</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Numero</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Bairro</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Cidade</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Cep</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Destinatário</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Endereco</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Origem_Geo</t>
         </is>
@@ -522,10 +534,10 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>-22.0856768</v>
+        <v>-22.084585</v>
       </c>
       <c r="J2" t="n">
-        <v>-48.7526652</v>
+        <v>-48.7532208</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -631,7 +643,7 @@
         <v>-22.0815719</v>
       </c>
       <c r="J4" t="n">
-        <v>-48.7476383</v>
+        <v>-48.7476382</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1064,49 +1076,49 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">MARCELA FERNANDA FAXINA DOS SANTOS </t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Rua João Francisco Pizato</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>110</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Parque Residencial Vila Rica</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Dois Córregos</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>17300188</t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">MARCELA FERNANDA FAXINA DOS SANTOS </t>
         </is>
       </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Rua João Francisco Pizzato, 110, Parque Residencial Vila Rica, Dois Córregos - SP</t>
         </is>
       </c>
-      <c r="I13" s="1" t="inlineStr"/>
-      <c r="J13" s="1" t="inlineStr"/>
-      <c r="K13" s="1" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Nao_Encontrado</t>
         </is>

</xml_diff>

<commit_message>
fix: remove neighborhood from Google Maps links
This introduces a new string builder formatting function specifically targeting maps URL links that skips including the neighborhood ("bairro") property. This ensures that clicking the final PDF link routes the user properly using just street name, number and city, while internal tools correctly keep using the full address format for accurate initial geocoding algorithm.

Co-authored-by: juniorchiodi <95029115+juniorchiodi@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ENDERECOS-ROTA.xlsx
+++ b/ENDERECOS-ROTA.xlsx
@@ -534,10 +534,10 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>-22.084585</v>
+        <v>-22.0884218</v>
       </c>
       <c r="J2" t="n">
-        <v>-48.7532208</v>
+        <v>-48.7510661</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -746,10 +746,10 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>-22.0867376</v>
+        <v>-22.0907603</v>
       </c>
       <c r="J6" t="n">
-        <v>-48.7506314</v>
+        <v>-48.7483911</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>

</xml_diff>